<commit_message>
Add Load Full Template page and clarify the minimum PMO
</commit_message>
<xml_diff>
--- a/example_data/PMO_building_template.xlsx
+++ b/example_data/PMO_building_template.xlsx
@@ -9,8 +9,8 @@
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Panel Targets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Genome Info" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Microhaplotype" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Microhaplotype" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Genome Info" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Specimen Level" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Project Info" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Library Sample Info" sheetId="7" state="visible" r:id="rId7"/>
@@ -238,7 +238,7 @@
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Index (starting at 0) of the genome in the Genome Info sheet that the genomic locations refer to. Defaults to 0 if left blank.</t>
+        <t>Optional. The genome in the Genome Info sheet that the genomic locations refer to, given as its name or its index (starting at 0). Defaults to the first genome if left blank.</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
@@ -328,35 +328,130 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Required. Name of the genome.</t>
+        <t>Required. A unique identifier for this sequencing/amplification run of a specimen.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Required. The NCBI taxonomy number.</t>
+        <t>Required. A name for this target.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Required. The genome version.</t>
+        <t>Required. The microhaplotype sequence.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Required. A link to where this genome file can be downloaded.</t>
+        <t>Required. The read count for this microhaplotype.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. A link to where this genome's annotation file can be downloaded.</t>
+        <t>Optional. The unique molecular identifier (UMI) count for this microhaplotype.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The chromosomes/contigs found within this genome.</t>
+        <t>Optional. The chromosome name.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Genomic start of the microhaplotype (0-based).</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Genomic end of the microhaplotype (0-based).</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. The reference sequence of this genomic location.</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Which strand the location is on: + or -.</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Additional annotations associated with this microhaplotype, e.g. wildtype.</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Start position(s) of masked segments within the sequence. Separate multiple values with commas.</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Size(s) of the masked segments. Separate multiple values with commas, in the same order as masking_seq_start.</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Size(s) of the replacement for each masked segment. Separate multiple values with commas, in the same order as masking_seq_start.</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. An optional name for this microhaplotype.</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. The pseudocigar of the microhaplotype. Requires pseudocigar_start and pseudocigar_end.</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Chromosome of the reference location the pseudocigar is relative to. Defaults to chrom if left blank.</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Start of the reference location the pseudocigar is relative to (0-based). Required if pseudocigar is given.</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. End of the reference location the pseudocigar is relative to (0-based). Required if pseudocigar is given.</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Reference sequence of the location the pseudocigar is relative to.</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Strand of the reference location the pseudocigar is relative to: + or -.</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. How the pseudocigar was generated.</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. The ASCII FASTQ per-base quality string for this sequence; must be the same length as the sequence.</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Extra information to store with the representative microhaplotype.</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Extra information to store with the detected microhaplotype.</t>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Custom. Fields not yet defined by the PMO schema that you want to include with your data. Rename this column (and add more) as needed.</t>
       </text>
@@ -373,130 +468,35 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Required. A unique identifier for this sequencing/amplification run of a specimen.</t>
+        <t>Required. Name of the genome.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
-        <t>Required. A name for this target.</t>
+        <t>Required. The NCBI taxonomy number.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Required. The microhaplotype sequence.</t>
+        <t>Required. The genome version.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Required. The read count for this microhaplotype.</t>
+        <t>Required. A link to where this genome file can be downloaded.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The unique molecular identifier (UMI) count for this microhaplotype.</t>
+        <t>Optional. A link to where this genome's annotation file can be downloaded.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The chromosome name.</t>
+        <t>Optional. The chromosomes/contigs found within this genome.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Genomic start of the microhaplotype (0-based).</t>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Genomic end of the microhaplotype (0-based).</t>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. The reference sequence of this genomic location.</t>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Which strand the location is on: + or -.</t>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Additional annotations associated with this microhaplotype, e.g. wildtype.</t>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Start position(s) of masked segments within the sequence. Separate multiple values with commas.</t>
-      </text>
-    </comment>
-    <comment ref="M1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Size(s) of the masked segments. Separate multiple values with commas, in the same order as masking_seq_start.</t>
-      </text>
-    </comment>
-    <comment ref="N1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Size(s) of the replacement for each masked segment. Separate multiple values with commas, in the same order as masking_seq_start.</t>
-      </text>
-    </comment>
-    <comment ref="O1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. An optional name for this microhaplotype.</t>
-      </text>
-    </comment>
-    <comment ref="P1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. The pseudocigar of the microhaplotype. Requires pseudocigar_start and pseudocigar_end.</t>
-      </text>
-    </comment>
-    <comment ref="Q1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Chromosome of the reference location the pseudocigar is relative to. Defaults to chrom if left blank.</t>
-      </text>
-    </comment>
-    <comment ref="R1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Start of the reference location the pseudocigar is relative to (0-based). Required if pseudocigar is given.</t>
-      </text>
-    </comment>
-    <comment ref="S1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. End of the reference location the pseudocigar is relative to (0-based). Required if pseudocigar is given.</t>
-      </text>
-    </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Reference sequence of the location the pseudocigar is relative to.</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Strand of the reference location the pseudocigar is relative to: + or -.</t>
-      </text>
-    </comment>
-    <comment ref="V1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. How the pseudocigar was generated.</t>
-      </text>
-    </comment>
-    <comment ref="W1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. The ASCII FASTQ per-base quality string for this sequence; must be the same length as the sequence.</t>
-      </text>
-    </comment>
-    <comment ref="X1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Extra information to store with the representative microhaplotype.</t>
-      </text>
-    </comment>
-    <comment ref="Y1" authorId="0" shapeId="0">
-      <text>
-        <t>Optional. Extra information to store with the detected microhaplotype.</t>
-      </text>
-    </comment>
-    <comment ref="Z1" authorId="0" shapeId="0">
       <text>
         <t>Custom. Fields not yet defined by the PMO schema that you want to include with your data. Rename this column (and add more) as needed.</t>
       </text>
@@ -523,27 +523,27 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The NCBI taxonomy number of the organism(s) in the specimen. Separate multiple values with commas for mixed samples.</t>
+        <t>Optional. The NCBI taxonomy number of the organism(s) in the specimen. Separate multiple values with commas for mixed samples. If included, fill in for every specimen.</t>
       </text>
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The NCBI taxonomy number of the host the specimen was collected from.</t>
+        <t>Optional. The NCBI taxonomy number of the host the specimen was collected from. If included, fill in for every specimen.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The date of specimen collection: YYYY, YYYY-MM, or YYYY-MM-DD.</t>
+        <t>Optional. The date of specimen collection: YYYY, YYYY-MM, or YYYY-MM-DD. If included, fill in for every specimen.</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. The country the specimen was collected in (admin level 0).</t>
+        <t>Optional. The country the specimen was collected in (admin level 0). If included, fill in for every specimen.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. A name for the project; must be unique if multiple projects are listed.</t>
+        <t>Optional. A name for the project; must be unique if multiple projects are listed. On the Specimen Level sheet, must match a project on the Project Info sheet and, if included, be filled in for every specimen.</t>
       </text>
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
@@ -698,7 +698,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Required. A name for the project; must be unique if multiple projects are listed.</t>
+        <t>Required. A name for the project; must be unique if multiple projects are listed. On the Specimen Level sheet, must match a project on the Project Info sheet and, if included, be filled in for every specimen.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -808,7 +808,7 @@
     </comment>
     <comment ref="N1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. A name for a specific sequencing run, e.g. batch1; must match a name in the Sequencing Info sheet.</t>
+        <t>Optional. A name for a specific sequencing run, e.g. batch1; must match a name in the Sequencing Info sheet. If included, fill in for every library sample.</t>
       </text>
     </comment>
     <comment ref="O1" authorId="0" shapeId="0">
@@ -828,7 +828,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>Required. A name for a specific sequencing run, e.g. batch1; must match a name in the Sequencing Info sheet.</t>
+        <t>Required. A name for a specific sequencing run, e.g. batch1; must match a name in the Sequencing Info sheet. If included, fill in for every library sample.</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -933,6 +933,11 @@
     </comment>
     <comment ref="C1" authorId="0" shapeId="0">
       <text>
+        <t>Optional. Name of the pipeline. On the Bioinformatics Methods sheet, rows with the same name form one pipeline; on the Bioinformatics Run sheet, the pipeline used for that run. Leave blank if there is only one pipeline.</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
         <t>Custom. Fields not yet defined by the PMO schema that you want to include with your data. Rename this column (and add more) as needed.</t>
       </text>
     </comment>
@@ -972,6 +977,11 @@
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Optional. Name of the pipeline. On the Bioinformatics Methods sheet, rows with the same name form one pipeline; on the Bioinformatics Run sheet, the pipeline used for that run. Leave blank if there is only one pipeline.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
       <text>
         <t>Custom. Fields not yet defined by the PMO schema that you want to include with your data. Rename this column (and add more) as needed.</t>
       </text>
@@ -1269,7 +1279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1302,117 +1312,102 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Each sheet is one table. Required columns must be completed to create a valid PMO; optional columns store additional metadata. Hover over a column header to see a description of the field.</t>
+          <t>A minimum PMO only needs the Panel Targets and Microhaplotype sheets (yellow-green tabs). All other sheets (pink tabs) are optional, but add context that makes the data easier to interpret and share; Specimen Level is highly recommended.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Column names match the PMO Builder app and the table-to-PMO functions in pmotools-python, so a completed sheet can be uploaded to the matching page of the app (select the sheet after uploading this workbook) or passed directly to pmotools-python.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
+          <t>Each sheet is one table. Required columns must be completed to create a valid PMO; optional columns store additional metadata. Hover over a column header to see a description of the field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Column names match the PMO Builder app and the table-to-PMO functions in pmotools-python. Upload the completed workbook on the app's Load Full Template page to load every sheet at once, upload it on a single page and select the matching sheet, or pass a sheet directly to pmotools-python. Sheets you leave empty are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
           <t>Some values are entered in the app rather than in a sheet: the panel name (Panel Information page) and the bioinformatics run name (Microhaplotype Information and Read Counts per Stage pages).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Columns that accept several values (noted in the header description) should be separated with commas. Dates should be stored as YYYY-MM-DD.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>You may add your own custom fields to store project-specific information. If there are fields you use regularly and believe would be broadly useful, please contact us so we can consider them for a future version of the PMO specification.</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Colour Key</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="n"/>
-      <c r="B11" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" t="inlineStr">
         <is>
           <t>Required in format</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" t="inlineStr">
         <is>
           <t>Not required in format</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Not defined by schema (custom fields are allowed, but not recommended)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>App page</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Associated PMO sections</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Panel Targets</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Panel Information</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>One row per target in the panel, with its primers and optional genomic locations. The panel name is entered in the app.</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>panel_info, target_info</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Genome Info</t>
+          <t>Panel Targets</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1422,12 +1417,12 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>The genome(s) the panel targets. Required if Panel Targets includes genomic locations.</t>
+          <t>One row per target in the panel, with its primers and optional genomic locations. The panel name is entered in the app.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>targeted_genomes</t>
+          <t>panel_info, target_info</t>
         </is>
       </c>
     </row>
@@ -1456,117 +1451,117 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Specimen Level</t>
+          <t>Genome Info</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Specimen Level Metadata</t>
+          <t>Panel Information</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Metadata on each biological specimen.</t>
+          <t>The genome(s) the panel targets. Required if Panel Targets includes genomic locations.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>specimen_info</t>
+          <t>targeted_genomes</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Project Info</t>
+          <t>Specimen Level</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Project Information</t>
+          <t>Specimen Level Metadata</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>The project(s) the specimens belong to.</t>
+          <t>Metadata on each biological specimen.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>project_info</t>
+          <t>specimen_info</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Library Sample Info</t>
+          <t>Project Info</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Library Sample Level Metadata</t>
+          <t>Project Information</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Each library prepared from a specimen; a specimen may have several library samples.</t>
+          <t>The project(s) the specimens belong to.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>library_sample_info</t>
+          <t>project_info</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Sequencing Info</t>
+          <t>Library Sample Info</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Sequencing Information</t>
+          <t>Library Sample Level Metadata</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>How the samples were sequenced, e.g. platform, instrument and dates.</t>
+          <t>Each library prepared from a specimen; a specimen may have several library samples.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>sequencing_info</t>
+          <t>library_sample_info</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Bioinformatics Run</t>
+          <t>Sequencing Info</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Bioinformatics Information</t>
+          <t>Sequencing Information</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Each bioinformatics run, if samples were analysed in one or several runs.</t>
+          <t>How the samples were sequenced, e.g. platform, instrument and dates.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>bioinformatics_run_info</t>
+          <t>sequencing_info</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Bioinformatics Methods</t>
+          <t>Bioinformatics Run</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1576,62 +1571,85 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>The programs used to generate the microhaplotypes.</t>
+          <t>Each bioinformatics run, if samples were analysed in one or several runs.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>bioinformatics_methods_info</t>
+          <t>bioinformatics_run_info</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Raw Read Counts</t>
+          <t>Bioinformatics Methods</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Read Counts per Stage</t>
+          <t>Bioinformatics Information</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Total raw read count for each library sample.</t>
+          <t>The programs used to generate the microhaplotypes, one row per program. Rows sharing a bioinformatics_method_name form one pipeline.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>read_counts_by_stage</t>
+          <t>bioinformatics_methods_info</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>Raw Read Counts</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Read Counts per Stage</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Total raw read count for each library sample.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>read_counts_by_stage</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>Reads by Stage</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Read Counts per Stage</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Read counts per library sample, per target, at each pipeline stage.</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>read_counts_by_stage</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A9:D9"/>
     <mergeCell ref="A8:D8"/>
     <mergeCell ref="A6:D6"/>
     <mergeCell ref="A4:D4"/>
@@ -1646,10 +1664,11 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1657,7 +1676,8 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1686,7 +1706,12 @@
           <t>program_url</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>bioinformatics_method_name</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>custom_field</t>
         </is>
@@ -1701,6 +1726,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1738,6 +1764,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1787,6 +1814,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00DDEE3B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1908,67 +1936,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="B1" s="4" t="inlineStr">
-        <is>
-          <t>taxon_id</t>
-        </is>
-      </c>
-      <c r="C1" s="4" t="inlineStr">
-        <is>
-          <t>genome_version</t>
-        </is>
-      </c>
-      <c r="D1" s="4" t="inlineStr">
-        <is>
-          <t>url</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>gff_url</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>chromosomes</t>
-        </is>
-      </c>
-      <c r="G1" s="6" t="inlineStr">
-        <is>
-          <t>custom_field</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
+    <tabColor rgb="00DDEE3B"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2141,9 +2109,72 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>taxon_id</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>genome_version</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>url</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>gff_url</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>chromosomes</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>custom_field</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2373,6 +2404,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2434,6 +2466,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2543,6 +2576,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -2664,15 +2698,17 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00FCDAE6"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2686,7 +2722,12 @@
           <t>run_date</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>bioinformatics_method_name</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>custom_field</t>
         </is>

</xml_diff>